<commit_message>
Updated validation for negative test data
</commit_message>
<xml_diff>
--- a/rules/CORE-000185/negative/01/data/unit-test-coreid-CG0123-negative.xlsx
+++ b/rules/CORE-000185/negative/01/data/unit-test-coreid-CG0123-negative.xlsx
@@ -36,7 +36,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -53,12 +53,6 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <b/>
     </font>
     <font>
       <sz val="11"/>
@@ -73,12 +67,8 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -91,23 +81,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
-        <bgColor/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <bgColor/>
       </patternFill>
     </fill>
@@ -137,17 +117,15 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,10 +468,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>3-4</v>
       </c>
     </row>
@@ -517,10 +495,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>dm.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Demographics</v>
       </c>
     </row>
@@ -533,7 +511,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -555,9 +533,49 @@
         <v>Error value</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C2" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D2" s="2">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="str">
+        <v>ACTARMCD</v>
+      </c>
+      <c r="F2" s="2" t="str">
+        <v>THIS IS LONGER THAN 20 CHARACTERS</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>dm.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Record</v>
+      </c>
+      <c r="D3" s="2">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>ACTARMCD</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>THIS IS LONGER THAN 20 CHARACTERS</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -597,10 +615,10 @@
       <c r="J1" s="3" t="str">
         <v>RFPENDTC</v>
       </c>
-      <c r="K1" s="4" t="str">
+      <c r="K1" s="3" t="str">
         <v>DTHDTC</v>
       </c>
-      <c r="L1" s="4" t="str">
+      <c r="L1" s="3" t="str">
         <v>DTHFL</v>
       </c>
       <c r="M1" s="3" t="str">
@@ -627,16 +645,16 @@
       <c r="T1" s="3" t="str">
         <v>ARMCD</v>
       </c>
-      <c r="U1" s="4" t="str">
+      <c r="U1" s="3" t="str">
         <v>ARM</v>
       </c>
       <c r="V1" s="3" t="str">
         <v>ACTARMCD</v>
       </c>
-      <c r="W1" s="5" t="str">
+      <c r="W1" s="3" t="str">
         <v>ACTARM</v>
       </c>
-      <c r="X1" s="4" t="str">
+      <c r="X1" s="3" t="str">
         <v>ARMNRS</v>
       </c>
       <c r="Y1" s="3" t="str">
@@ -647,564 +665,564 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="str">
+      <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="6" t="str">
+      <c r="B2" s="5" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="6" t="str">
+      <c r="C2" s="5" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="6" t="str">
+      <c r="D2" s="5" t="str">
         <v>Subject Identifier for the Study</v>
       </c>
-      <c r="E2" s="6" t="str">
+      <c r="E2" s="5" t="str">
         <v>Subject Reference Start Date/Time</v>
       </c>
-      <c r="F2" s="6" t="str">
+      <c r="F2" s="5" t="str">
         <v>Subject Reference End Date/Time</v>
       </c>
-      <c r="G2" s="6" t="str">
+      <c r="G2" s="5" t="str">
         <v>Date/Time of First Study Treatment</v>
       </c>
-      <c r="H2" s="6" t="str">
+      <c r="H2" s="5" t="str">
         <v>Date/Time of Last Study Treatment</v>
       </c>
-      <c r="I2" s="6" t="str">
+      <c r="I2" s="5" t="str">
         <v>Date/Time of Informed Consent</v>
       </c>
-      <c r="J2" s="6" t="str">
+      <c r="J2" s="5" t="str">
         <v>Date/Time of End of Participation</v>
       </c>
-      <c r="K2" s="6" t="str">
+      <c r="K2" s="5" t="str">
         <v>Date/Time of Death</v>
       </c>
-      <c r="L2" s="6" t="str">
+      <c r="L2" s="5" t="str">
         <v>Subject Death Flag</v>
       </c>
-      <c r="M2" s="6" t="str">
+      <c r="M2" s="5" t="str">
         <v>Study Site Identifier</v>
       </c>
-      <c r="N2" s="6" t="str">
+      <c r="N2" s="5" t="str">
         <v>Date/Time of Birth</v>
       </c>
-      <c r="O2" s="6" t="str">
+      <c r="O2" s="5" t="str">
         <v>Age</v>
       </c>
-      <c r="P2" s="6" t="str">
+      <c r="P2" s="5" t="str">
         <v>Age Units</v>
       </c>
-      <c r="Q2" s="6" t="str">
+      <c r="Q2" s="5" t="str">
         <v>Sex</v>
       </c>
-      <c r="R2" s="6" t="str">
+      <c r="R2" s="5" t="str">
         <v>Race</v>
       </c>
-      <c r="S2" s="6" t="str">
+      <c r="S2" s="5" t="str">
         <v>Ethnicity</v>
       </c>
-      <c r="T2" s="6" t="str">
+      <c r="T2" s="5" t="str">
         <v>Planned Arm Code</v>
       </c>
-      <c r="U2" s="6" t="str">
+      <c r="U2" s="5" t="str">
         <v>Description of Planned Arm</v>
       </c>
-      <c r="V2" s="6" t="str">
+      <c r="V2" s="5" t="str">
         <v>Actual Arm Code</v>
       </c>
-      <c r="W2" s="6" t="str">
+      <c r="W2" s="5" t="str">
         <v>Description of Actual Arm</v>
       </c>
-      <c r="X2" s="6" t="str">
+      <c r="X2" s="5" t="str">
         <v>Reason Arm and/or Actual Arm is Null</v>
       </c>
-      <c r="Y2" s="6" t="str">
+      <c r="Y2" s="5" t="str">
         <v>Description of Unplanned Actual Arm</v>
       </c>
-      <c r="Z2" s="6" t="str">
+      <c r="Z2" s="5" t="str">
         <v>Country</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="6" t="str">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="5" t="str">
         <v>Num</v>
       </c>
-      <c r="P3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Y3" s="6" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="6" t="str">
+      <c r="P3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Y3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6">
+      <c r="A4" s="5">
         <v>12</v>
       </c>
-      <c r="B4" s="6">
+      <c r="B4" s="5">
         <v>2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>20</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="5">
         <v>12</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="5">
         <v>10</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="5">
         <v>10</v>
       </c>
-      <c r="G4" s="6">
+      <c r="G4" s="5">
         <v>10</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>10</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>10</v>
       </c>
-      <c r="J4" s="6">
+      <c r="J4" s="5">
         <v>10</v>
       </c>
-      <c r="K4" s="6">
+      <c r="K4" s="5">
         <v>10</v>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="5">
         <v>1</v>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="5">
         <v>3</v>
       </c>
-      <c r="N4" s="6">
+      <c r="N4" s="5">
         <v>10</v>
       </c>
-      <c r="O4" s="6">
+      <c r="O4" s="5">
         <v>8</v>
       </c>
-      <c r="P4" s="6">
+      <c r="P4" s="5">
         <v>5</v>
       </c>
-      <c r="Q4" s="6">
+      <c r="Q4" s="5">
         <v>1</v>
       </c>
-      <c r="R4" s="6">
+      <c r="R4" s="5">
         <v>41</v>
       </c>
-      <c r="S4" s="6">
+      <c r="S4" s="5">
         <v>22</v>
       </c>
-      <c r="T4" s="6">
+      <c r="T4" s="5">
         <v>8</v>
       </c>
-      <c r="U4" s="6">
+      <c r="U4" s="5">
         <v>28</v>
       </c>
-      <c r="V4" s="6" t="str">
+      <c r="V4" s="5" t="str">
         <v>20</v>
       </c>
-      <c r="W4" s="6">
+      <c r="W4" s="5">
         <v>28</v>
       </c>
-      <c r="X4" s="6">
+      <c r="X4" s="5">
         <v>14</v>
       </c>
-      <c r="Y4" s="6">
+      <c r="Y4" s="5">
         <v>200</v>
       </c>
-      <c r="Z4" s="6">
+      <c r="Z4" s="5">
         <v>3</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="str">
+      <c r="A5" s="4" t="str">
         <v>CDISCCORE01</v>
       </c>
-      <c r="B5" s="7" t="str">
+      <c r="B5" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C5" s="7" t="str">
+      <c r="C5" s="4" t="str">
         <v>015246-099-0000-00000</v>
       </c>
-      <c r="D5" s="7" t="str">
+      <c r="D5" s="4" t="str">
         <v>099000000000</v>
       </c>
-      <c r="E5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="F5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="I5" s="7" t="str">
+      <c r="E5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I5" s="4" t="str">
         <v>2018-04-16</v>
       </c>
-      <c r="J5" s="7" t="str">
+      <c r="J5" s="4" t="str">
         <v>2018-05-04</v>
       </c>
-      <c r="K5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="L5" s="7" t="str">
+      <c r="K5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="M5" s="7" t="str">
+      <c r="M5" s="4" t="str">
         <v>0990000</v>
       </c>
-      <c r="N5" s="7" t="str">
+      <c r="N5" s="4" t="str">
         <v>1940-08-14</v>
       </c>
-      <c r="O5" s="7" t="str">
+      <c r="O5" s="4" t="str">
         <v>77</v>
       </c>
-      <c r="P5" s="7" t="str">
+      <c r="P5" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q5" s="7" t="str">
+      <c r="Q5" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R5" s="7" t="str">
+      <c r="R5" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S5" s="7" t="str">
+      <c r="S5" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="U5" s="7" t="str">
+      <c r="T5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U5" s="4" t="str">
         <v>IKd</v>
       </c>
-      <c r="V5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="W5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="X5" s="7" t="str">
+      <c r="V5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X5" s="4" t="str">
         <v>ASSIGNED, NOT TREATED</v>
       </c>
-      <c r="Y5" s="7" t="str">
-        <v/>
-      </c>
-      <c r="Z5" s="7" t="str">
+      <c r="Y5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z5" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="str">
+      <c r="A6" s="4" t="str">
         <v>CDISCCORE01</v>
       </c>
-      <c r="B6" s="7" t="str">
+      <c r="B6" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C6" s="7" t="str">
+      <c r="C6" s="4" t="str">
         <v>015246-099-0000-00001</v>
       </c>
-      <c r="D6" s="7" t="str">
+      <c r="D6" s="4" t="str">
         <v>099000000001</v>
       </c>
-      <c r="E6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="F6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="I6" s="7" t="str">
+      <c r="E6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I6" s="4" t="str">
         <v>2018-05-20</v>
       </c>
-      <c r="J6" s="7" t="str">
+      <c r="J6" s="4" t="str">
         <v>2018-06-10</v>
       </c>
-      <c r="K6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="L6" s="7" t="str">
+      <c r="K6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L6" s="4" t="str">
         <v>U</v>
       </c>
-      <c r="M6" s="7" t="str">
+      <c r="M6" s="4" t="str">
         <v>0990000</v>
       </c>
-      <c r="N6" s="7" t="str">
+      <c r="N6" s="4" t="str">
         <v>1941-08-14</v>
       </c>
-      <c r="O6" s="7" t="str">
+      <c r="O6" s="4" t="str">
         <v>76</v>
       </c>
-      <c r="P6" s="7" t="str">
+      <c r="P6" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q6" s="7" t="str">
+      <c r="Q6" s="4" t="str">
         <v>M</v>
       </c>
-      <c r="R6" s="7" t="str">
+      <c r="R6" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S6" s="7" t="str">
+      <c r="S6" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="U6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="V6" s="8" t="str">
+      <c r="T6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="V6" s="6" t="str">
         <v>THIS IS LONGER THAN 20 CHARACTERS</v>
       </c>
-      <c r="W6" s="8" t="str">
+      <c r="W6" s="4" t="str">
         <v>IKD</v>
       </c>
-      <c r="X6" s="7" t="str">
+      <c r="X6" s="4" t="str">
         <v>NOT ASSIGNED</v>
       </c>
-      <c r="Y6" s="7" t="str">
-        <v/>
-      </c>
-      <c r="Z6" s="7" t="str">
+      <c r="Y6" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z6" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
-      <c r="A7" s="7" t="str">
+      <c r="A7" s="4" t="str">
         <v>CDISCCORE01</v>
       </c>
-      <c r="B7" s="7" t="str">
+      <c r="B7" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C7" s="7" t="str">
+      <c r="C7" s="4" t="str">
         <v>015246-099-0000-00002</v>
       </c>
-      <c r="D7" s="7" t="str">
+      <c r="D7" s="4" t="str">
         <v>099000000002</v>
       </c>
-      <c r="E7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="F7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="G7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="H7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="I7" s="7" t="str">
+      <c r="E7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I7" s="4" t="str">
         <v>2018-05-20</v>
       </c>
-      <c r="J7" s="7" t="str">
+      <c r="J7" s="4" t="str">
         <v>2018-06-10</v>
       </c>
-      <c r="K7" s="7" t="str">
+      <c r="K7" s="4" t="str">
         <v>2018-06-10</v>
       </c>
-      <c r="L7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="M7" s="7" t="str">
+      <c r="L7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M7" s="4" t="str">
         <v>0990000</v>
       </c>
-      <c r="N7" s="7" t="str">
+      <c r="N7" s="4" t="str">
         <v>1942-08-14</v>
       </c>
-      <c r="O7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="P7" s="7" t="str">
+      <c r="O7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P7" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q7" s="7" t="str">
+      <c r="Q7" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R7" s="7" t="str" xml:space="preserve">
+      <c r="R7" s="4" t="str" xml:space="preserve">
         <v xml:space="preserve">BLACK OR
 AFRICAN
 AMERICAN</v>
       </c>
-      <c r="S7" s="7" t="str">
+      <c r="S7" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="U7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="V7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="W7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="X7" s="7" t="str">
+      <c r="T7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="V7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X7" s="4" t="str">
         <v>SCREEN FAILURE</v>
       </c>
-      <c r="Y7" s="7" t="str">
-        <v/>
-      </c>
-      <c r="Z7" s="7" t="str">
+      <c r="Y7" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z7" s="4" t="str">
         <v>USA</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="str">
+      <c r="A8" s="4" t="str">
         <v>CDISCCORE01</v>
       </c>
-      <c r="B8" s="9" t="str">
+      <c r="B8" s="4" t="str">
         <v>DM</v>
       </c>
-      <c r="C8" s="7" t="str">
+      <c r="C8" s="4" t="str">
         <v>015246-099-0000-00003</v>
       </c>
-      <c r="D8" s="7" t="str">
+      <c r="D8" s="4" t="str">
         <v>099000000003</v>
       </c>
-      <c r="E8" s="9" t="str">
+      <c r="E8" s="4" t="str">
         <v>2018-05-08T11:20</v>
       </c>
-      <c r="F8" s="9" t="str">
+      <c r="F8" s="4" t="str">
         <v>2018-08-29T10:35</v>
       </c>
-      <c r="G8" s="9" t="str">
+      <c r="G8" s="4" t="str">
         <v>2018-05-08T11:20</v>
       </c>
-      <c r="H8" s="9" t="str">
+      <c r="H8" s="4" t="str">
         <v>2018-08-29T10:35</v>
       </c>
-      <c r="I8" s="9" t="str">
+      <c r="I8" s="4" t="str">
         <v>2018-04-17</v>
       </c>
-      <c r="J8" s="9" t="str">
+      <c r="J8" s="4" t="str">
         <v>2018-09-04</v>
       </c>
-      <c r="K8" s="7" t="str">
+      <c r="K8" s="4" t="str">
         <v>2018-09-04</v>
       </c>
-      <c r="L8" s="7" t="str">
+      <c r="L8" s="4" t="str">
         <v>N</v>
       </c>
-      <c r="M8" s="7" t="str">
+      <c r="M8" s="4" t="str">
         <v>0990000</v>
       </c>
-      <c r="N8" s="9" t="str">
+      <c r="N8" s="4" t="str">
         <v>1947-12-23</v>
       </c>
-      <c r="O8" s="7" t="str">
+      <c r="O8" s="4" t="str">
         <v>70</v>
       </c>
-      <c r="P8" s="7" t="str">
+      <c r="P8" s="4" t="str">
         <v>YEARS</v>
       </c>
-      <c r="Q8" s="9" t="str">
+      <c r="Q8" s="4" t="str">
         <v>F</v>
       </c>
-      <c r="R8" s="9" t="str">
+      <c r="R8" s="4" t="str">
         <v>WHITE</v>
       </c>
-      <c r="S8" s="9" t="str">
+      <c r="S8" s="4" t="str">
         <v>NOT HISPANIC OR LATINO</v>
       </c>
-      <c r="T8" s="7" t="str">
+      <c r="T8" s="4" t="str">
         <v>IKD</v>
       </c>
-      <c r="U8" s="7" t="str">
+      <c r="U8" s="4" t="str">
         <v>IKd</v>
       </c>
-      <c r="V8" s="9" t="str">
+      <c r="V8" s="7" t="str">
         <v>THIS IS LONGER THAN 20 CHARACTERS</v>
       </c>
-      <c r="W8" s="7" t="str">
+      <c r="W8" s="4" t="str">
         <v>Placebo</v>
       </c>
-      <c r="X8" s="7" t="str">
+      <c r="X8" s="4" t="str">
         <v>UNPLANNED TREATMENT</v>
       </c>
-      <c r="Y8" s="9" t="str">
-        <v/>
-      </c>
-      <c r="Z8" s="9" t="str">
+      <c r="Y8" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z8" s="4" t="str">
         <v>GRC</v>
       </c>
     </row>

</xml_diff>